<commit_message>
Add validator, e2e flows, request generator modules; fix template_flow propagation in Pass-validation assertions
- Fix missing template_flow argument on assert_error_doesnt_exist calls in
  utils/allure_wrapper.py so PRE_TEMPLATE.* variables resolve correctly for
  "Pass validation" test cases (previously only assert_error_exists passed it)
- Add new asserter/validator modules (error_text_processor, validator/,
  report_row_type, response_codes) and reporting utilities (ado_reporter,
  azure_reporting, csv_custom_report, dependency_tracker, iris_db)
- Add e2e flows, request generator, and database GUI tabs
- Add CI pipeline config (azure-pipelines.yml, .github/workflows) and docs
- Add new/updated XML request templates and test resources

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/Service-Codes.xlsx
+++ b/resources/Service-Codes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BaraaAlmousa\Documents\projects\clone project\sff-demo-1-enhance\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BaraaAlmousa\Documents\projects\clone project\sff-demo\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B62A21D-52B4-49D1-A3AD-394CA6F593F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE86CD40-4104-47FA-8530-8834167A55AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5E6711D2-B9D7-49E8-B85D-7AE59811DC01}"/>
+    <workbookView xWindow="-3105" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{5E6711D2-B9D7-49E8-B85D-7AE59811DC01}"/>
   </bookViews>
   <sheets>
     <sheet name="SERVICE" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="408">
   <si>
     <t>Emergency Room - Hourly Rate</t>
   </si>
@@ -59,12 +59,6 @@
     <t>51-03</t>
   </si>
   <si>
-    <t>Undefined services</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
     <t>Comprehensive screening evaluation and management by clinician of an individual, including an age and gender appropriate history, questionnaire filling, examination, and ordering of laboratory/diagnostic procedures, new or established patient; 30-40 minutes.</t>
   </si>
   <si>
@@ -135,18 +129,6 @@
   </si>
   <si>
     <t>20-03</t>
-  </si>
-  <si>
-    <t>Consultation - GP - Follow Up within one week</t>
-  </si>
-  <si>
-    <t>9.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Room and Board: Private Room Deluxe </t>
-  </si>
-  <si>
-    <t>17-08</t>
   </si>
   <si>
     <t>Room Rate difference - Daily Rate  (Day 1 and more  ) - Isolation Room</t>
@@ -260,18 +242,6 @@
     <t>51-02</t>
   </si>
   <si>
-    <t>Room and Board/ Perdiem - Category 18</t>
-  </si>
-  <si>
-    <t>17-18</t>
-  </si>
-  <si>
-    <t>Perdiem - Day Stay (Day Care) Room  - NOT inclusive of Laboratory and Radiology</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
     <t>Perdiem - Short Stay</t>
   </si>
   <si>
@@ -296,12 +266,6 @@
     <t>17-22</t>
   </si>
   <si>
-    <t>Perdiem - Treatment or Observation Room - NOT inclusive of Laboratory and Radiology</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
     <t xml:space="preserve">Room Rate difference - Daily Rate  (Day 1 and more ) - Suite  </t>
   </si>
   <si>
@@ -324,12 +288,6 @@
   </si>
   <si>
     <t>20-02</t>
-  </si>
-  <si>
-    <t>Consultation - Consultant - Follow Up within one week</t>
-  </si>
-  <si>
-    <t>11.1</t>
   </si>
   <si>
     <t>Perdiem - SCU - Daily Rate (Day 4 to 8)</t>
@@ -354,24 +312,983 @@
   </si>
   <si>
     <t>Type</t>
+  </si>
+  <si>
+    <t>14-01</t>
+  </si>
+  <si>
+    <t>14-02</t>
+  </si>
+  <si>
+    <t>14-03</t>
+  </si>
+  <si>
+    <t>17-02</t>
+  </si>
+  <si>
+    <t>17-03</t>
+  </si>
+  <si>
+    <t>17-05</t>
+  </si>
+  <si>
+    <t>17-06</t>
+  </si>
+  <si>
+    <t>17-07-01</t>
+  </si>
+  <si>
+    <t>17-07-02</t>
+  </si>
+  <si>
+    <t>17-07-03</t>
+  </si>
+  <si>
+    <t>17-11-2</t>
+  </si>
+  <si>
+    <t>17-12-01</t>
+  </si>
+  <si>
+    <t>17-14</t>
+  </si>
+  <si>
+    <t>17-16</t>
+  </si>
+  <si>
+    <t>17-23</t>
+  </si>
+  <si>
+    <t>17-25</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>18-02</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>19-01</t>
+  </si>
+  <si>
+    <t>19-02</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>20-01</t>
+  </si>
+  <si>
+    <t>20-04</t>
+  </si>
+  <si>
+    <t>20-05</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>3-02</t>
+  </si>
+  <si>
+    <t>3-03</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>4-01</t>
+  </si>
+  <si>
+    <t>4-02</t>
+  </si>
+  <si>
+    <t>4-03</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>50-02</t>
+  </si>
+  <si>
+    <t>50-03</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>01-10</t>
+  </si>
+  <si>
+    <t>01-11-01</t>
+  </si>
+  <si>
+    <t>01-11-02</t>
+  </si>
+  <si>
+    <t>01-11-03</t>
+  </si>
+  <si>
+    <t>01-11-04</t>
+  </si>
+  <si>
+    <t>08-01</t>
+  </si>
+  <si>
+    <t>08-02</t>
+  </si>
+  <si>
+    <t>08-03</t>
+  </si>
+  <si>
+    <t>08-04</t>
+  </si>
+  <si>
+    <t>08-05</t>
+  </si>
+  <si>
+    <t>08-06</t>
+  </si>
+  <si>
+    <t>08-07</t>
+  </si>
+  <si>
+    <t>08-08</t>
+  </si>
+  <si>
+    <t>08-09</t>
+  </si>
+  <si>
+    <t>17-25-1</t>
+  </si>
+  <si>
+    <t>17-25-2</t>
+  </si>
+  <si>
+    <t>17-25-3</t>
+  </si>
+  <si>
+    <t>17-25-4</t>
+  </si>
+  <si>
+    <t>17-25-5</t>
+  </si>
+  <si>
+    <t>17-26-1</t>
+  </si>
+  <si>
+    <t>17-26-2</t>
+  </si>
+  <si>
+    <t>17-26-3</t>
+  </si>
+  <si>
+    <t>17-26-4</t>
+  </si>
+  <si>
+    <t>17-26-5</t>
+  </si>
+  <si>
+    <t>17-27</t>
+  </si>
+  <si>
+    <t>17-27-1</t>
+  </si>
+  <si>
+    <t>17-27-2</t>
+  </si>
+  <si>
+    <t>17-27-3</t>
+  </si>
+  <si>
+    <t>17-28</t>
+  </si>
+  <si>
+    <t>17-29</t>
+  </si>
+  <si>
+    <t>17-40</t>
+  </si>
+  <si>
+    <t>22-01</t>
+  </si>
+  <si>
+    <t>22-02</t>
+  </si>
+  <si>
+    <t>22-03</t>
+  </si>
+  <si>
+    <t>22-04</t>
+  </si>
+  <si>
+    <t>22-05</t>
+  </si>
+  <si>
+    <t>22-06</t>
+  </si>
+  <si>
+    <t>22-07</t>
+  </si>
+  <si>
+    <t>22-08</t>
+  </si>
+  <si>
+    <t>52-21</t>
+  </si>
+  <si>
+    <t>52-22</t>
+  </si>
+  <si>
+    <t>52-23</t>
+  </si>
+  <si>
+    <t>52-24</t>
+  </si>
+  <si>
+    <t>52-25</t>
+  </si>
+  <si>
+    <t>52-26</t>
+  </si>
+  <si>
+    <t>52-27</t>
+  </si>
+  <si>
+    <t>52-28</t>
+  </si>
+  <si>
+    <t>52-29</t>
+  </si>
+  <si>
+    <t>52-30</t>
+  </si>
+  <si>
+    <t>52-31</t>
+  </si>
+  <si>
+    <t>52-32</t>
+  </si>
+  <si>
+    <t>52-33</t>
+  </si>
+  <si>
+    <t>52-34</t>
+  </si>
+  <si>
+    <t>52-35</t>
+  </si>
+  <si>
+    <t>52-36</t>
+  </si>
+  <si>
+    <t>52-37</t>
+  </si>
+  <si>
+    <t>52-38</t>
+  </si>
+  <si>
+    <t>52-39</t>
+  </si>
+  <si>
+    <t>52-40</t>
+  </si>
+  <si>
+    <t>53-01</t>
+  </si>
+  <si>
+    <t>53-03</t>
+  </si>
+  <si>
+    <t>53-04</t>
+  </si>
+  <si>
+    <t>53-05</t>
+  </si>
+  <si>
+    <t>54-01</t>
+  </si>
+  <si>
+    <t>54-02</t>
+  </si>
+  <si>
+    <t>54-03</t>
+  </si>
+  <si>
+    <t>54-04</t>
+  </si>
+  <si>
+    <t>55-01</t>
+  </si>
+  <si>
+    <t>55-02</t>
+  </si>
+  <si>
+    <t>55-03</t>
+  </si>
+  <si>
+    <t>55-04</t>
+  </si>
+  <si>
+    <t>55-05</t>
+  </si>
+  <si>
+    <t>56-01</t>
+  </si>
+  <si>
+    <t>56-02</t>
+  </si>
+  <si>
+    <t>56-03</t>
+  </si>
+  <si>
+    <t>57-02</t>
+  </si>
+  <si>
+    <t>57-03</t>
+  </si>
+  <si>
+    <t>57-04</t>
+  </si>
+  <si>
+    <t>57-05</t>
+  </si>
+  <si>
+    <t>57-06</t>
+  </si>
+  <si>
+    <t>58-02</t>
+  </si>
+  <si>
+    <t>58-03</t>
+  </si>
+  <si>
+    <t>58-05</t>
+  </si>
+  <si>
+    <t>59-02</t>
+  </si>
+  <si>
+    <t>59-03</t>
+  </si>
+  <si>
+    <t>59-04</t>
+  </si>
+  <si>
+    <t>59-06</t>
+  </si>
+  <si>
+    <t>59-07</t>
+  </si>
+  <si>
+    <t>59-08</t>
+  </si>
+  <si>
+    <t>59-10</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>70-01</t>
+  </si>
+  <si>
+    <t>70-02</t>
+  </si>
+  <si>
+    <t>70-03</t>
+  </si>
+  <si>
+    <t>70-04</t>
+  </si>
+  <si>
+    <t>70-05</t>
+  </si>
+  <si>
+    <t>70-06</t>
+  </si>
+  <si>
+    <t>70-07</t>
+  </si>
+  <si>
+    <t>70-08</t>
+  </si>
+  <si>
+    <t>70-09</t>
+  </si>
+  <si>
+    <t>70-10</t>
+  </si>
+  <si>
+    <t>70-11</t>
+  </si>
+  <si>
+    <t>70-12</t>
+  </si>
+  <si>
+    <t>70-13</t>
+  </si>
+  <si>
+    <t>70-14</t>
+  </si>
+  <si>
+    <t>70-15</t>
+  </si>
+  <si>
+    <t>70-16</t>
+  </si>
+  <si>
+    <t>70-17</t>
+  </si>
+  <si>
+    <t>70-18</t>
+  </si>
+  <si>
+    <t>70-19</t>
+  </si>
+  <si>
+    <t>70-20</t>
+  </si>
+  <si>
+    <t>70-21</t>
+  </si>
+  <si>
+    <t>70-22</t>
+  </si>
+  <si>
+    <t>88</t>
+  </si>
+  <si>
+    <t>97</t>
+  </si>
+  <si>
+    <t>98</t>
+  </si>
+  <si>
+    <t>Perdiem - Haemodialysis  (HD)</t>
+  </si>
+  <si>
+    <t>Perdiem - Automated Peritoneal Dialysis (APD).</t>
+  </si>
+  <si>
+    <t>Perdiem - Continuous  Ambulatory Peritoneal Dialysis (CAPD).</t>
+  </si>
+  <si>
+    <t>Room and Board:  VIP Room</t>
+  </si>
+  <si>
+    <t>Room and Board: First Class Room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Room and Board: Ward </t>
+  </si>
+  <si>
+    <t>Room and Board: Royal Suite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - PICU - Daily Rate (Day 8 to 14) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - PICU - Daily Rate (Day 15 to 21) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - PICU - Daily Rate  (Day 22 and more) </t>
+  </si>
+  <si>
+    <t>Perdiem - International Assistance in case of Emergency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - New-born Nursery  -  Daily Rate (Day 4 to 8) </t>
+  </si>
+  <si>
+    <t>Perdiem - Long Term Stay - Daily Rate - Intermediate Cases</t>
+  </si>
+  <si>
+    <t>Perdiem - Long Term Stay - Daily Rate - Severe Cases</t>
+  </si>
+  <si>
+    <t>Recovery Room  - Hourly Rate</t>
+  </si>
+  <si>
+    <t>Day Stay (Day care) Room - Daily Rate</t>
+  </si>
+  <si>
+    <t>Perdiem - SCU - Daily Rate (Day 1 to 3)</t>
+  </si>
+  <si>
+    <t>Perdiem - SCU - Daily Rate (Day 9 and more)</t>
+  </si>
+  <si>
+    <t>Perdiem - SCBU  - Daily Rate (Day 1 to 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - SCBU  - Daily Rate (Day 4 to 8) </t>
+  </si>
+  <si>
+    <t>Perdiem - SCBU  - Daily Rate  (Day 9 and more)</t>
+  </si>
+  <si>
+    <t>Perdiem  - Ward or Shared Room - Daily Rate (Day 4 to 8)</t>
+  </si>
+  <si>
+    <t>Operating Room Services - Minor Surgery</t>
+  </si>
+  <si>
+    <t>Catheterization Lab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery Room </t>
+  </si>
+  <si>
+    <t>Perdiem - Companion Accommodation</t>
+  </si>
+  <si>
+    <t>Intensive Care Unit (ICU)</t>
+  </si>
+  <si>
+    <t>Perdiem  - Ward or Shared Room - Daily Rate  (Day 8 and more)</t>
+  </si>
+  <si>
+    <t>Special Care Baby Unit (SCBU)</t>
+  </si>
+  <si>
+    <t>Room Rate difference - Daily Rate  (Day 1 and more ) - VIP Room</t>
+  </si>
+  <si>
+    <t>Room Rate difference - Daily Rate   (Day 1 and more  ) - First Class Room</t>
+  </si>
+  <si>
+    <t>Paediatric intensive care Unit (PICU)</t>
+  </si>
+  <si>
+    <t>Nursery - General Classification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - ICU/CCU - Daily Rate (Day 1 to 7) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - ICU/CCU - Daily Rate (Day 8 to 14) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - ICU/CCU - Daily Rate (Day 15 to 21) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - ICU/CCU - Daily Rate (Day 22 and more) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - NICU - Daily Rate (Day 1 to 7) </t>
+  </si>
+  <si>
+    <t>Comprehensive screening by a non-physician clinician of an individual, including vital signs, an age and gender appropriate history, coordination for ordering of laboratory/diagnostic procedures and questionnaire filling, new or established patient; 30-40 minutes.</t>
+  </si>
+  <si>
+    <t>Educational services rendered by Clinician (Physician or Non-Physician) to patient opting out of the  Comprehensive Screening, new or established patient; 10-15 minutes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - NICU - Daily Rate (Day 15 to 21) </t>
+  </si>
+  <si>
+    <t>Medicine Home Delivery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perdiem - NICU - Daily Rate (Day 22 and more) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nurse lead Pfizer COVID-19 Vaccine administration </t>
+  </si>
+  <si>
+    <t>Physician teleconsultation during Coronavirus disease (COVID-19) vaccine administration</t>
+  </si>
+  <si>
+    <t>Teleconsultation for International patient care (IPC) including medical doctor to medical doctor &amp; patient, each 20 minutes</t>
+  </si>
+  <si>
+    <t>Teleconsultation for International patient care (IPC), multidisciplinary team &amp; patient, primary provider, each 20 minutes</t>
+  </si>
+  <si>
+    <t>Teleconsultation for International patient care (IPC), multidisciplinary team &amp; patient, each additional provider, each 20 minutes</t>
+  </si>
+  <si>
+    <t>Teleconsultation for International patient care (IPC), medical doctor to medical doctor</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 0 – 6 years for initial visit</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 0 – 6 years for minimum requirement of dental services for Quarter 1 to Quarter 3 from initiation (each quarter)</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 0 – 6 years for minimum requirement of dental services for Quarter 4 from initiation</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 7 – 12 years for initial visit</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 7 – 12 years for minimum requirement of dental services for Quarter 1 to Quarter 3 from initiation (each quarter)</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 7 – 12 years for minimum requirement of dental services for Quarter 4 from initiation</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 13 – 17 years for initial visit</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 13 – 17 years for minimum requirement of dental services for Quarter 1 to Quarter 3 from initiation (each quarter)</t>
+  </si>
+  <si>
+    <t>Dental Capitation package for children age 13 – 17 years for minimum requirement of dental services for Quarter 4 from initiation</t>
+  </si>
+  <si>
+    <t>Per Diem- Simple Home Visit - Nursing Service
+Includes all medical services and transportation
+Excludes medication, consumables and equipment</t>
+  </si>
+  <si>
+    <t>Per Diem- Simple Home Visit - Supportive Service ( Physiotherapy, Speech Therapy, Occupational Therapy, Respiratory Therapy)
+Includes all medical services and transportation
+Excludes medication, consumables and equipment</t>
+  </si>
+  <si>
+    <t>Per Diem- Specialized Home Visit - Consultation by Specialty Physician or Psychotherapy services
+Includes all medical services and transportation
+Excludes medication, consumables and equipment</t>
+  </si>
+  <si>
+    <t>Per Diem- Routine Home Nursing Care
+Includes all medical services and transportation
+Excludes medication, consumables and equipment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per Diem- Advanced Home Nursing Care
+Includes all medical services and transportation
+Excludes medication, consumables and equipment </t>
+  </si>
+  <si>
+    <t>Per Diem- Bundled Base Payment of home care (Level 1- SIMPLE )                                                                                                                    * -A bundled payment that includes all medical services and transportation - Supportive services: includes Physiotherapy, Speech Therapy, Occupational Therapy, Respiratory Therapy - bundled payment excludes medication, consumables and equipment which will be paid separately</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per Diem- Bundled Base Payment of home care  (Level 2- Intermediate )                                                                                                           * -A bundled payment that includes all medical services and transportation - Supportive services: includes Physiotherapy, Speech Therapy, Occupational Therapy, Respiratory Therapy - bundled payment excludes medication, consumables and equipment which will be paid separately </t>
+  </si>
+  <si>
+    <t>Per Diem-  Bundled Base Payment of home care  (Level 3- Intensive)                                                                                                                              * -A bundled payment that includes all medical services and transportation - Supportive services: includes Physiotherapy, Speech Therapy, Occupational Therapy, Respiratory Therapy - bundled payment excludes medication, consumables and equipment which will be paid separately</t>
+  </si>
+  <si>
+    <t>Per Diem- Bundled Base Payment of home care  (Level 4- Complex )                                                                                                                     *-A bundled payment that includes all medical services and transportation - Supportive services: includes Physiotherapy, Speech Therapy, Occupational Therapy, Respiratory Therapy - bundled payment excludes medication, consumables and equipment which will be paid separately</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COVID-19 Home Isolation &amp; Home quarantine programs Home visit </t>
+  </si>
+  <si>
+    <t>Transferred non ventilated LTC patient due to COVID-19 measures from SEHA to other facilities</t>
+  </si>
+  <si>
+    <t>Tele consultation – Consultant /  specialist - Home isolation for asymptomatic COVID-19 patients or with mild symptoms out of healthcare facilities and provide care for them at home</t>
+  </si>
+  <si>
+    <t>Tele consultation – Nurse assessment - Home isolation for asymptomatic COVID-19 patients or with mild symptoms out of healthcare facilities and provide care for them at home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tele consultation – Nurse assessment – Population  at risk program to provide care at home  </t>
+  </si>
+  <si>
+    <t>Transferred  ventilated LTC patient due to COVID-19 measures from SEHA to other facilities</t>
+  </si>
+  <si>
+    <t>Transferred non ventilated LTC patient due to COVID-19 measures from SEHA to other facilities with post acute rehabilitation (PAR)</t>
+  </si>
+  <si>
+    <t>Transferred  ventilated LTC patient due to COVID-19 measures from SEHA to other facilities with post acute rehabilitation (PAR)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Pre-transplantation work-up (Autologous)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Preparation (Autologous)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Transplantation (Autologous)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Post-transplantation follow-up (Autologous)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Pre-transplantation work-up (Allogenic)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Preparation (Allogenic)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Transplantation (Allogenic)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Bone Marrow Post-transplantation follow-up (Allogenic)</t>
+  </si>
+  <si>
+    <t>Comprehensive Screening Major Package for male &amp; female (age 18-39 years)</t>
+  </si>
+  <si>
+    <t>Comprehensive Screening Major Package for male &amp; female (age 40-64 years)</t>
+  </si>
+  <si>
+    <t>Comprehensive Screening Major Package for male &amp; female (age 65-75 years)</t>
+  </si>
+  <si>
+    <t>Comprehensive Screening Minor Package for male &amp; female (age 65-75 years) for Vision Screening</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comprehensive Screening Oral Health Package for male &amp; female (age 18-75 years) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon Cancer Screening male &amp; female (age 40-75 years) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cervical Cancer Screening for female (age 25-29 years) </t>
+  </si>
+  <si>
+    <t>Cervical Cancer Screening for female (age 30-65 years) for eligible groups based on PCSP standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lung Cancer Screening for (High Risk) male &amp; female (age 55-75 years) </t>
+  </si>
+  <si>
+    <t>Standalone Screening Mammography for female for eligible groups based on PCSP standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standalone Screening Fecal immunochemical test (FIT) for eligible groups based on PCSP standard </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standalone Screening Abdominal Aortic Aneurysm for eligible groups based on PCSP standard </t>
+  </si>
+  <si>
+    <t>Standalone Screening DEXA scan for eligible groups based on PCSP standard</t>
+  </si>
+  <si>
+    <t>Standalone Screening Liquid Biopsy for Colorectal Cancer</t>
+  </si>
+  <si>
+    <t>Comprehensive Screening Minor Package for Male &amp; Female (Age 50-64 years) for Hearing and Dementia Screening</t>
+  </si>
+  <si>
+    <t>Comprehensive Screening Minor Package for Male &amp; Female (Age 65-75 years) for Hearing and Dementia Screening</t>
+  </si>
+  <si>
+    <t>Standalone Screening for Breast Cancer for Female (Age 20-34 Years)</t>
+  </si>
+  <si>
+    <t>Standalone Screening for Breast Cancer for Female with Gail Risk Assessment (Age 35-39 Years)</t>
+  </si>
+  <si>
+    <t>Reproductive Health Screening for Female (Age 20-35 years)</t>
+  </si>
+  <si>
+    <t>Reproductive Health Screening for Male (Age 20-35 years)</t>
+  </si>
+  <si>
+    <t>Genetic testing for Pre – Marital Screening, includes analysis and reporting of 569 genes</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Testicular Tissue Cryopreservation</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Ovarian Tissue Cryopreservation</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Histotripsy Treatment</t>
+  </si>
+  <si>
+    <t>Biobanking; Umbilical Cord Blood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biobanking; Body Fluids </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biobanking; Human Tissue </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biobanking; Human DNA  </t>
+  </si>
+  <si>
+    <t>Ambulance service, Non- Critical transport, (BLS)</t>
+  </si>
+  <si>
+    <t>Ambulance service, advanced life support, Critical  transport, (ALS)</t>
+  </si>
+  <si>
+    <t>Specialty Care Transport</t>
+  </si>
+  <si>
+    <t>Neonatal Transport Ambulance</t>
+  </si>
+  <si>
+    <t>Ground mileage, per Kilometer</t>
+  </si>
+  <si>
+    <t>Ambulance service, Non- Critical Transport, (BLS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specialty care Transport  </t>
+  </si>
+  <si>
+    <t>Apheresis procedure Day 1</t>
+  </si>
+  <si>
+    <t>Apheresis procedure Day 2</t>
+  </si>
+  <si>
+    <t>Conditioning Journey</t>
+  </si>
+  <si>
+    <t>CART Infusion , Post CAR –T Care &amp; Complications</t>
+  </si>
+  <si>
+    <t>CART Follow Ups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundled Reimbursement for RBC Exchange Pre-Mobilization for Casgevy Treatment </t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Stem Cell Mobilization for Casgevy Treatment of Sickle Cell Anemia Patients</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Stem Cell Mobilization Days 5-6 for Casgevy Treatment of Thalassemia Patients</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Lymph Node Bio-bridge Anastomosis</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Lymph Node Transfer with Free Lymph Node Flap</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Lymph Node Transfer with Free Omental Flap</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Lymph Venous Anastomosis</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Lymphedema Debulking with Lipectomy and Split Thickness Skin Graft</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for Lymphedema Lymphatic Sparing Liposuction</t>
+  </si>
+  <si>
+    <t>Bundled Reimbursement for each additional site(limb) treated with any of the Lymphedema Surgical Interventions</t>
+  </si>
+  <si>
+    <t>Retinal screening Artificial Intelligence  (AI)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for completed regular ART cycle</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for embryo(s) storage</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for completed ART cycle from frozen embryo(s)</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for egg(s) storage</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Completed ART cycle from frozen egg(s)</t>
+  </si>
+  <si>
+    <t>Stimulation of ovaries</t>
+  </si>
+  <si>
+    <t>Egg retrieval</t>
+  </si>
+  <si>
+    <t>Egg freezing</t>
+  </si>
+  <si>
+    <t>Fertilization of eggs</t>
+  </si>
+  <si>
+    <t>Embryo freezing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add-on Fertility Investigation </t>
+  </si>
+  <si>
+    <t>Pre-implantation genetic testing for aneuploidy (PGT-A)</t>
+  </si>
+  <si>
+    <t>PGT-A for each additional embryo</t>
+  </si>
+  <si>
+    <t>Pre-implantation genetic testing for monogenic gene disorders (PGT-M)</t>
+  </si>
+  <si>
+    <t>PGT-M for each additional embryo</t>
+  </si>
+  <si>
+    <t>Pre-implantation genetic for structural chromosomal rearrangements (PGT-SR)</t>
+  </si>
+  <si>
+    <t>PGT-SR for each additional embryo</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for Micro-TESE</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for TESE</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for TESA</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for PESA</t>
+  </si>
+  <si>
+    <t>Bundled reimbursement for MESA</t>
+  </si>
+  <si>
+    <t>Outlier Payment "See Home care Standard'</t>
+  </si>
+  <si>
+    <t>Coronavirus disease (COVID-19) Vaccine administration outside healthcare facilities.</t>
+  </si>
+  <si>
+    <t>DRG Add-on Payment for High Cost Consumables</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -382,7 +1299,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -390,30 +1307,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,6 +1328,18 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E7663B41-1C57-49FF-B7C0-13755583A007}" name="Table1" displayName="Table1" ref="A1:C204" totalsRowShown="0" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:C204" xr:uid="{E7663B41-1C57-49FF-B7C0-13755583A007}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{75E782B9-94EF-4126-B1BF-AC6C1702F973}" name="Type" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{93F60A15-DBDC-4692-9E0D-82F7BB08249B}" name="Code" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{2D74B1F3-BB14-4EB3-B8A7-56E37AC67C2D}" name="Code Description" dataCellStyle="Normal"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -716,18 +1627,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D7E9D6-C55A-4751-98E4-60E31EF028ED}">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C204"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="255.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>101</v>
+      <c r="A1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -735,10 +1649,10 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -746,10 +1660,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -757,10 +1671,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -768,10 +1682,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -779,10 +1693,10 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -790,10 +1704,10 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -801,10 +1715,10 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -812,10 +1726,10 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -823,10 +1737,10 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>83</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -834,10 +1748,10 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -845,10 +1759,10 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="C12" t="s">
-        <v>79</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -856,10 +1770,10 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -867,10 +1781,10 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -878,10 +1792,10 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -889,10 +1803,10 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -900,10 +1814,10 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -911,10 +1825,10 @@
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -922,10 +1836,10 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -933,10 +1847,10 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>259</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -944,10 +1858,10 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -955,10 +1869,10 @@
         <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="C22" t="s">
-        <v>59</v>
+        <v>260</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -966,10 +1880,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -977,10 +1891,10 @@
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -988,10 +1902,10 @@
         <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="C25" t="s">
-        <v>53</v>
+        <v>261</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -999,10 +1913,10 @@
         <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1010,10 +1924,10 @@
         <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
+        <v>103</v>
       </c>
       <c r="C27" t="s">
-        <v>49</v>
+        <v>262</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1021,10 +1935,10 @@
         <v>2</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1032,10 +1946,10 @@
         <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="C29" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1043,10 +1957,10 @@
         <v>2</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>43</v>
+        <v>263</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1054,10 +1968,10 @@
         <v>2</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C31" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1065,10 +1979,10 @@
         <v>2</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>105</v>
       </c>
       <c r="C32" t="s">
-        <v>39</v>
+        <v>264</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1076,10 +1990,10 @@
         <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="C33" t="s">
-        <v>37</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1087,10 +2001,10 @@
         <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="C34" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1098,10 +2012,10 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>34</v>
+        <v>106</v>
       </c>
       <c r="C35" t="s">
-        <v>33</v>
+        <v>265</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1109,10 +2023,10 @@
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="C36" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1120,10 +2034,10 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="C37" t="s">
-        <v>29</v>
+        <v>266</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1131,10 +2045,10 @@
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>28</v>
+        <v>108</v>
       </c>
       <c r="C38" t="s">
-        <v>27</v>
+        <v>267</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1142,10 +2056,10 @@
         <v>2</v>
       </c>
       <c r="B39" t="s">
-        <v>26</v>
+        <v>109</v>
       </c>
       <c r="C39" t="s">
-        <v>25</v>
+        <v>268</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1153,10 +2067,10 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>24</v>
+        <v>110</v>
       </c>
       <c r="C40" t="s">
-        <v>23</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1164,10 +2078,10 @@
         <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>22</v>
+        <v>111</v>
       </c>
       <c r="C41" t="s">
-        <v>21</v>
+        <v>270</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1175,10 +2089,10 @@
         <v>2</v>
       </c>
       <c r="B42" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C42" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1186,10 +2100,10 @@
         <v>2</v>
       </c>
       <c r="B43" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
       <c r="C43" t="s">
-        <v>17</v>
+        <v>271</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1197,10 +2111,10 @@
         <v>2</v>
       </c>
       <c r="B44" t="s">
-        <v>16</v>
+        <v>82</v>
       </c>
       <c r="C44" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1208,10 +2122,10 @@
         <v>2</v>
       </c>
       <c r="B45" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C45" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1219,10 +2133,10 @@
         <v>2</v>
       </c>
       <c r="B46" t="s">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>272</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1230,10 +2144,10 @@
         <v>2</v>
       </c>
       <c r="B47" t="s">
-        <v>10</v>
+        <v>114</v>
       </c>
       <c r="C47" t="s">
-        <v>9</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1241,10 +2155,10 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="C48" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1252,10 +2166,10 @@
         <v>2</v>
       </c>
       <c r="B49" t="s">
-        <v>6</v>
+        <v>78</v>
       </c>
       <c r="C49" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1263,10 +2177,10 @@
         <v>2</v>
       </c>
       <c r="B50" t="s">
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="C50" t="s">
-        <v>3</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1274,13 +2188,1699 @@
         <v>2</v>
       </c>
       <c r="B51" t="s">
-        <v>1</v>
+        <v>115</v>
       </c>
       <c r="C51" t="s">
-        <v>0</v>
+        <v>274</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>2</v>
+      </c>
+      <c r="B52" t="s">
+        <v>116</v>
+      </c>
+      <c r="C52" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>2</v>
+      </c>
+      <c r="B53" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>2</v>
+      </c>
+      <c r="B54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>2</v>
+      </c>
+      <c r="B55" t="s">
+        <v>48</v>
+      </c>
+      <c r="C55" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>2</v>
+      </c>
+      <c r="B56" t="s">
+        <v>117</v>
+      </c>
+      <c r="C56" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>118</v>
+      </c>
+      <c r="C57" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>76</v>
+      </c>
+      <c r="C58" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>119</v>
+      </c>
+      <c r="C59" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>120</v>
+      </c>
+      <c r="C60" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>2</v>
+      </c>
+      <c r="B61" t="s">
+        <v>38</v>
+      </c>
+      <c r="C61" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>2</v>
+      </c>
+      <c r="B62" t="s">
+        <v>121</v>
+      </c>
+      <c r="C62" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>2</v>
+      </c>
+      <c r="B63" t="s">
+        <v>32</v>
+      </c>
+      <c r="C63" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>2</v>
+      </c>
+      <c r="B64" t="s">
+        <v>122</v>
+      </c>
+      <c r="C64" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s">
+        <v>123</v>
+      </c>
+      <c r="C65" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>2</v>
+      </c>
+      <c r="B66" t="s">
+        <v>124</v>
+      </c>
+      <c r="C66" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" t="s">
+        <v>125</v>
+      </c>
+      <c r="C67" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B68" t="s">
+        <v>126</v>
+      </c>
+      <c r="C68" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>2</v>
+      </c>
+      <c r="B69" t="s">
+        <v>127</v>
+      </c>
+      <c r="C69" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>2</v>
+      </c>
+      <c r="B70" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>2</v>
+      </c>
+      <c r="B71" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>2</v>
+      </c>
+      <c r="B72" t="s">
+        <v>129</v>
+      </c>
+      <c r="C72" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>2</v>
+      </c>
+      <c r="B73" t="s">
+        <v>58</v>
+      </c>
+      <c r="C73" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>2</v>
+      </c>
+      <c r="B74" t="s">
+        <v>66</v>
+      </c>
+      <c r="C74" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>2</v>
+      </c>
+      <c r="B75" t="s">
+        <v>6</v>
+      </c>
+      <c r="C75" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>2</v>
+      </c>
+      <c r="B76" t="s">
+        <v>64</v>
+      </c>
+      <c r="C76" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>2</v>
+      </c>
+      <c r="B77" t="s">
+        <v>130</v>
+      </c>
+      <c r="C77" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>2</v>
+      </c>
+      <c r="B78" t="s">
+        <v>131</v>
+      </c>
+      <c r="C78" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>2</v>
+      </c>
+      <c r="B79" t="s">
+        <v>132</v>
+      </c>
+      <c r="C79" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>2</v>
+      </c>
+      <c r="B80" t="s">
+        <v>36</v>
+      </c>
+      <c r="C80" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>2</v>
+      </c>
+      <c r="B81">
+        <v>96</v>
+      </c>
+      <c r="C81" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>2</v>
+      </c>
+      <c r="B82" t="s">
+        <v>133</v>
+      </c>
+      <c r="C82" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>2</v>
+      </c>
+      <c r="B83" t="s">
+        <v>134</v>
+      </c>
+      <c r="C83" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>2</v>
+      </c>
+      <c r="B84" t="s">
+        <v>135</v>
+      </c>
+      <c r="C84" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>2</v>
+      </c>
+      <c r="B85" t="s">
+        <v>136</v>
+      </c>
+      <c r="C85" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>2</v>
+      </c>
+      <c r="B86" t="s">
+        <v>137</v>
+      </c>
+      <c r="C86" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>2</v>
+      </c>
+      <c r="B87" t="s">
+        <v>138</v>
+      </c>
+      <c r="C87" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>2</v>
+      </c>
+      <c r="B88" t="s">
+        <v>139</v>
+      </c>
+      <c r="C88" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>2</v>
+      </c>
+      <c r="B89" t="s">
+        <v>140</v>
+      </c>
+      <c r="C89" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>2</v>
+      </c>
+      <c r="B90" t="s">
+        <v>141</v>
+      </c>
+      <c r="C90" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>2</v>
+      </c>
+      <c r="B91" t="s">
+        <v>142</v>
+      </c>
+      <c r="C91" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>2</v>
+      </c>
+      <c r="B92" t="s">
+        <v>143</v>
+      </c>
+      <c r="C92" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>2</v>
+      </c>
+      <c r="B93" t="s">
+        <v>144</v>
+      </c>
+      <c r="C93" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>2</v>
+      </c>
+      <c r="B94" t="s">
+        <v>145</v>
+      </c>
+      <c r="C94" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>2</v>
+      </c>
+      <c r="B95" t="s">
+        <v>146</v>
+      </c>
+      <c r="C95" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>2</v>
+      </c>
+      <c r="B96" t="s">
+        <v>147</v>
+      </c>
+      <c r="C96" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>2</v>
+      </c>
+      <c r="B97" t="s">
+        <v>148</v>
+      </c>
+      <c r="C97" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>2</v>
+      </c>
+      <c r="B98" t="s">
+        <v>149</v>
+      </c>
+      <c r="C98" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>2</v>
+      </c>
+      <c r="B99" t="s">
+        <v>150</v>
+      </c>
+      <c r="C99" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>2</v>
+      </c>
+      <c r="B100" t="s">
+        <v>151</v>
+      </c>
+      <c r="C100" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>2</v>
+      </c>
+      <c r="B101" t="s">
+        <v>152</v>
+      </c>
+      <c r="C101" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>2</v>
+      </c>
+      <c r="B102" t="s">
+        <v>153</v>
+      </c>
+      <c r="C102" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>2</v>
+      </c>
+      <c r="B103" t="s">
+        <v>154</v>
+      </c>
+      <c r="C103" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>2</v>
+      </c>
+      <c r="B104" t="s">
+        <v>155</v>
+      </c>
+      <c r="C104" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>2</v>
+      </c>
+      <c r="B105" t="s">
+        <v>156</v>
+      </c>
+      <c r="C105" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>2</v>
+      </c>
+      <c r="B106" t="s">
+        <v>157</v>
+      </c>
+      <c r="C106" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>2</v>
+      </c>
+      <c r="B107" t="s">
+        <v>158</v>
+      </c>
+      <c r="C107" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>2</v>
+      </c>
+      <c r="B108" t="s">
+        <v>159</v>
+      </c>
+      <c r="C108" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>2</v>
+      </c>
+      <c r="B109" t="s">
+        <v>160</v>
+      </c>
+      <c r="C109" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>2</v>
+      </c>
+      <c r="B110" t="s">
+        <v>161</v>
+      </c>
+      <c r="C110" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>2</v>
+      </c>
+      <c r="B111" t="s">
+        <v>162</v>
+      </c>
+      <c r="C111" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>2</v>
+      </c>
+      <c r="B112" t="s">
+        <v>163</v>
+      </c>
+      <c r="C112" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>2</v>
+      </c>
+      <c r="B113" t="s">
+        <v>164</v>
+      </c>
+      <c r="C113" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>2</v>
+      </c>
+      <c r="B114" t="s">
+        <v>165</v>
+      </c>
+      <c r="C114" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>2</v>
+      </c>
+      <c r="B115" t="s">
+        <v>166</v>
+      </c>
+      <c r="C115" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>2</v>
+      </c>
+      <c r="B116" t="s">
+        <v>167</v>
+      </c>
+      <c r="C116" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>2</v>
+      </c>
+      <c r="B117" t="s">
+        <v>168</v>
+      </c>
+      <c r="C117" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>2</v>
+      </c>
+      <c r="B118" t="s">
+        <v>169</v>
+      </c>
+      <c r="C118" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>2</v>
+      </c>
+      <c r="B119" t="s">
+        <v>170</v>
+      </c>
+      <c r="C119" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>2</v>
+      </c>
+      <c r="B120" t="s">
+        <v>171</v>
+      </c>
+      <c r="C120" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>2</v>
+      </c>
+      <c r="B121" t="s">
+        <v>172</v>
+      </c>
+      <c r="C121" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>2</v>
+      </c>
+      <c r="B122" t="s">
+        <v>173</v>
+      </c>
+      <c r="C122" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>2</v>
+      </c>
+      <c r="B123" t="s">
+        <v>174</v>
+      </c>
+      <c r="C123" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>2</v>
+      </c>
+      <c r="B124" t="s">
+        <v>175</v>
+      </c>
+      <c r="C124" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>2</v>
+      </c>
+      <c r="B125" t="s">
+        <v>176</v>
+      </c>
+      <c r="C125" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>2</v>
+      </c>
+      <c r="B126" t="s">
+        <v>177</v>
+      </c>
+      <c r="C126" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>2</v>
+      </c>
+      <c r="B127" t="s">
+        <v>178</v>
+      </c>
+      <c r="C127" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>2</v>
+      </c>
+      <c r="B128" t="s">
+        <v>179</v>
+      </c>
+      <c r="C128" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>2</v>
+      </c>
+      <c r="B129" t="s">
+        <v>180</v>
+      </c>
+      <c r="C129" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>2</v>
+      </c>
+      <c r="B130" t="s">
+        <v>181</v>
+      </c>
+      <c r="C130" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>2</v>
+      </c>
+      <c r="B131" t="s">
+        <v>182</v>
+      </c>
+      <c r="C131" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>2</v>
+      </c>
+      <c r="B132" t="s">
+        <v>183</v>
+      </c>
+      <c r="C132" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>2</v>
+      </c>
+      <c r="B133" t="s">
+        <v>184</v>
+      </c>
+      <c r="C133" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>2</v>
+      </c>
+      <c r="B134" t="s">
+        <v>185</v>
+      </c>
+      <c r="C134" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>2</v>
+      </c>
+      <c r="B135" t="s">
+        <v>186</v>
+      </c>
+      <c r="C135" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>2</v>
+      </c>
+      <c r="B136" t="s">
+        <v>187</v>
+      </c>
+      <c r="C136" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>2</v>
+      </c>
+      <c r="B137" t="s">
+        <v>188</v>
+      </c>
+      <c r="C137" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>2</v>
+      </c>
+      <c r="B138" t="s">
+        <v>189</v>
+      </c>
+      <c r="C138" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B139" t="s">
+        <v>190</v>
+      </c>
+      <c r="C139" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>2</v>
+      </c>
+      <c r="B140" t="s">
+        <v>191</v>
+      </c>
+      <c r="C140" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>2</v>
+      </c>
+      <c r="B141" t="s">
+        <v>192</v>
+      </c>
+      <c r="C141" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>2</v>
+      </c>
+      <c r="B142" t="s">
+        <v>193</v>
+      </c>
+      <c r="C142" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>2</v>
+      </c>
+      <c r="B143" t="s">
+        <v>194</v>
+      </c>
+      <c r="C143" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>2</v>
+      </c>
+      <c r="B144" t="s">
+        <v>195</v>
+      </c>
+      <c r="C144" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>2</v>
+      </c>
+      <c r="B145" t="s">
+        <v>196</v>
+      </c>
+      <c r="C145" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>2</v>
+      </c>
+      <c r="B146" t="s">
+        <v>197</v>
+      </c>
+      <c r="C146" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>2</v>
+      </c>
+      <c r="B147" t="s">
+        <v>198</v>
+      </c>
+      <c r="C147" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>2</v>
+      </c>
+      <c r="B148" t="s">
+        <v>199</v>
+      </c>
+      <c r="C148" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>2</v>
+      </c>
+      <c r="B149" t="s">
+        <v>200</v>
+      </c>
+      <c r="C149" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>2</v>
+      </c>
+      <c r="B150" t="s">
+        <v>201</v>
+      </c>
+      <c r="C150" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>2</v>
+      </c>
+      <c r="B151" t="s">
+        <v>202</v>
+      </c>
+      <c r="C151" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>2</v>
+      </c>
+      <c r="B152" t="s">
+        <v>203</v>
+      </c>
+      <c r="C152" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>2</v>
+      </c>
+      <c r="B153" t="s">
+        <v>204</v>
+      </c>
+      <c r="C153" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>2</v>
+      </c>
+      <c r="B154" t="s">
+        <v>205</v>
+      </c>
+      <c r="C154" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>2</v>
+      </c>
+      <c r="B155" t="s">
+        <v>206</v>
+      </c>
+      <c r="C155" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>2</v>
+      </c>
+      <c r="B156" t="s">
+        <v>207</v>
+      </c>
+      <c r="C156" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>2</v>
+      </c>
+      <c r="B157" t="s">
+        <v>10</v>
+      </c>
+      <c r="C157" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>2</v>
+      </c>
+      <c r="B158" t="s">
+        <v>208</v>
+      </c>
+      <c r="C158" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>2</v>
+      </c>
+      <c r="B159" t="s">
+        <v>209</v>
+      </c>
+      <c r="C159" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>2</v>
+      </c>
+      <c r="B160" t="s">
+        <v>210</v>
+      </c>
+      <c r="C160" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>2</v>
+      </c>
+      <c r="B161" t="s">
+        <v>211</v>
+      </c>
+      <c r="C161" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>2</v>
+      </c>
+      <c r="B162" t="s">
+        <v>212</v>
+      </c>
+      <c r="C162" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>2</v>
+      </c>
+      <c r="B163" t="s">
+        <v>56</v>
+      </c>
+      <c r="C163" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>2</v>
+      </c>
+      <c r="B164" t="s">
+        <v>213</v>
+      </c>
+      <c r="C164" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>2</v>
+      </c>
+      <c r="B165" t="s">
+        <v>214</v>
+      </c>
+      <c r="C165" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>2</v>
+      </c>
+      <c r="B166" t="s">
+        <v>72</v>
+      </c>
+      <c r="C166" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>2</v>
+      </c>
+      <c r="B167" t="s">
+        <v>215</v>
+      </c>
+      <c r="C167" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>2</v>
+      </c>
+      <c r="B168" t="s">
+        <v>62</v>
+      </c>
+      <c r="C168" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>2</v>
+      </c>
+      <c r="B169" t="s">
+        <v>28</v>
+      </c>
+      <c r="C169" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>2</v>
+      </c>
+      <c r="B170" t="s">
+        <v>216</v>
+      </c>
+      <c r="C170" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>2</v>
+      </c>
+      <c r="B171" t="s">
+        <v>217</v>
+      </c>
+      <c r="C171" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>2</v>
+      </c>
+      <c r="B172" t="s">
+        <v>218</v>
+      </c>
+      <c r="C172" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>2</v>
+      </c>
+      <c r="B173" t="s">
+        <v>40</v>
+      </c>
+      <c r="C173" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>2</v>
+      </c>
+      <c r="B174" t="s">
+        <v>219</v>
+      </c>
+      <c r="C174" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>2</v>
+      </c>
+      <c r="B175" t="s">
+        <v>220</v>
+      </c>
+      <c r="C175" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>2</v>
+      </c>
+      <c r="B176" t="s">
+        <v>221</v>
+      </c>
+      <c r="C176" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>2</v>
+      </c>
+      <c r="B177" t="s">
+        <v>22</v>
+      </c>
+      <c r="C177" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>2</v>
+      </c>
+      <c r="B178" t="s">
+        <v>222</v>
+      </c>
+      <c r="C178" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>2</v>
+      </c>
+      <c r="B179" t="s">
+        <v>223</v>
+      </c>
+      <c r="C179" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>2</v>
+      </c>
+      <c r="B180" t="s">
+        <v>224</v>
+      </c>
+      <c r="C180" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>2</v>
+      </c>
+      <c r="B181" t="s">
+        <v>225</v>
+      </c>
+      <c r="C181" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>2</v>
+      </c>
+      <c r="B182" t="s">
+        <v>226</v>
+      </c>
+      <c r="C182" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>2</v>
+      </c>
+      <c r="B183" t="s">
+        <v>227</v>
+      </c>
+      <c r="C183" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>2</v>
+      </c>
+      <c r="B184" t="s">
+        <v>228</v>
+      </c>
+      <c r="C184" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>2</v>
+      </c>
+      <c r="B185" t="s">
+        <v>229</v>
+      </c>
+      <c r="C185" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>2</v>
+      </c>
+      <c r="B186" t="s">
+        <v>230</v>
+      </c>
+      <c r="C186" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>2</v>
+      </c>
+      <c r="B187" t="s">
+        <v>231</v>
+      </c>
+      <c r="C187" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>2</v>
+      </c>
+      <c r="B188" t="s">
+        <v>232</v>
+      </c>
+      <c r="C188" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>2</v>
+      </c>
+      <c r="B189" t="s">
+        <v>233</v>
+      </c>
+      <c r="C189" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>2</v>
+      </c>
+      <c r="B190" t="s">
+        <v>234</v>
+      </c>
+      <c r="C190" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>2</v>
+      </c>
+      <c r="B191" t="s">
+        <v>235</v>
+      </c>
+      <c r="C191" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>2</v>
+      </c>
+      <c r="B192" t="s">
+        <v>236</v>
+      </c>
+      <c r="C192" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>2</v>
+      </c>
+      <c r="B193" t="s">
+        <v>237</v>
+      </c>
+      <c r="C193" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>2</v>
+      </c>
+      <c r="B194" t="s">
+        <v>238</v>
+      </c>
+      <c r="C194" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>2</v>
+      </c>
+      <c r="B195" t="s">
+        <v>239</v>
+      </c>
+      <c r="C195" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>2</v>
+      </c>
+      <c r="B196" t="s">
+        <v>240</v>
+      </c>
+      <c r="C196" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>2</v>
+      </c>
+      <c r="B197" t="s">
+        <v>241</v>
+      </c>
+      <c r="C197" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>2</v>
+      </c>
+      <c r="B198" t="s">
+        <v>242</v>
+      </c>
+      <c r="C198" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>2</v>
+      </c>
+      <c r="B199" t="s">
+        <v>243</v>
+      </c>
+      <c r="C199" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>2</v>
+      </c>
+      <c r="B200" t="s">
+        <v>244</v>
+      </c>
+      <c r="C200" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>2</v>
+      </c>
+      <c r="B201" t="s">
+        <v>245</v>
+      </c>
+      <c r="C201" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>2</v>
+      </c>
+      <c r="B202" t="s">
+        <v>246</v>
+      </c>
+      <c r="C202" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>2</v>
+      </c>
+      <c r="B203" t="s">
+        <v>247</v>
+      </c>
+      <c r="C203" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>2</v>
+      </c>
+      <c r="B204" t="s">
+        <v>248</v>
+      </c>
+      <c r="C204" t="s">
+        <v>407</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>